<commit_message>
Custom Roles: prod-vs-staging compare — add intended-reduction (Yes/No) + spec-citation columns
QA-lead clarification: list EVERY prod>staging capability delta (staging has LESS
than prod), including spec-intended reductions — annotate instead of filter.

- PLAN §4: revised main-tab column list to 11 cols (adds 'Per spec - intended
  reduction? (Yes/No)' + 'Spec citation'); noted all prod>staging deltas listed;
  added Summary-tab per-role Yes/No breakdown (No's = headline release risks).
- gen_prod_vs_staging.py: added the two columns to the row schema + per-role
  Yes/No counts (+TOTAL row) on the Summary tab; READ ME banner note.
- Regenerated interim xlsx + md; prod cells still spec-predicted/NEEDS-REVIEW.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/custom-roles-run/Prod-vs-Staging-Permission-Gaps_2026-07-14.xlsx
+++ b/build/custom-roles-run/Prod-vs-Staging-Permission-Gaps_2026-07-14.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +45,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -72,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -80,6 +83,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -448,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -544,6 +548,44 @@
       <c r="A15" t="inlineStr">
         <is>
           <t>live, then re-run gen_prod_vs_staging.py with the prod capture wired in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EVERY prod&gt;staging delta is listed (staging has LESS than prod) - spec-intended</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>reductions are INCLUDED, annotated 'Per spec - intended reduction? (Yes/No)' with a</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>'Spec citation'. The 'No' rows (reductions NOT accounted for in the spec) are the</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>headline release risks. All interim deltas are Yes (spec-declared); No's may appear</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>once live production is captured. See the Summary tab for the per-role Yes/No counts.</t>
         </is>
       </c>
     </row>
@@ -558,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -566,10 +608,12 @@
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -600,22 +644,32 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Delta</t>
+          <t>Delta (PROD-ONLY / match / staging-more)</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
+          <t>Per spec - intended reduction? (Yes/No)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Spec citation</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>Confidence / Needs-review</t>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Evidence / source</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Confidence (live/spec-predicted/NEEDS-REVIEW)</t>
         </is>
       </c>
     </row>
@@ -652,17 +706,27 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Spec 'Behavior Changes for Migrating Users' table (updated-spec-source.md) - Service Manager: 'Loses Invoicing Delete (cannot reverse invoices)'</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Spec Behavior-Changes: Service Manager 'Loses Invoicing Delete (cannot reverse)'</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW - prod side unverified (no live prod data)</t>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>spec-predicted / NEEDS REVIEW - prod side unverified (no live prod data)</t>
         </is>
       </c>
     </row>
@@ -699,17 +763,27 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Spec 'Behavior Changes for Migrating Users' table - Service Manager: 'Loses Settings: Service'</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Spec Behavior-Changes: Service Manager 'Loses Settings: Service'</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW - prod side unverified (no live prod data)</t>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>spec-predicted / NEEDS REVIEW - prod side unverified (no live prod data)</t>
         </is>
       </c>
     </row>
@@ -746,17 +820,27 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Spec 'Behavior Changes for Migrating Users' table - Service Manager: 'Loses Settings: Parts'</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Spec Behavior-Changes: Service Manager 'Loses Settings: Parts'</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW - prod side unverified (no live prod data)</t>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>spec-predicted / NEEDS REVIEW - prod side unverified (no live prod data)</t>
         </is>
       </c>
     </row>
@@ -793,17 +877,27 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Spec 'Behavior Changes for Migrating Users' table - Service Manager: 'Loses Settings: Finance'</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Spec Behavior-Changes: Service Manager 'Loses Settings: Finance'</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW - prod side unverified (no live prod data)</t>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>spec-predicted / NEEDS REVIEW - prod side unverified (no live prod data)</t>
         </is>
       </c>
     </row>
@@ -840,17 +934,27 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Spec 'Behavior Changes for Migrating Users' table - Service Manager: 'Loses Settings: Data Import'</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Spec Behavior-Changes: Service Manager 'Loses Settings: Data Import'</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW - prod side unverified (no live prod data)</t>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>spec-predicted / NEEDS REVIEW - prod side unverified (no live prod data)</t>
         </is>
       </c>
     </row>
@@ -887,17 +991,27 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Spec 'Behavior Changes for Migrating Users' table - Foreman: 'Loses Timesheets Edit'</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Spec Behavior-Changes: Foreman 'Loses Timesheets Edit'</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW - prod side unverified (no live prod data)</t>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>spec-predicted / NEEDS REVIEW - prod side unverified (no live prod data)</t>
         </is>
       </c>
     </row>
@@ -934,17 +1048,27 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Spec 'Behavior Changes for Migrating Users' table - Technician: 'Loses Send to Portal'</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Spec Behavior-Changes: Technician 'Lose Send to Portal'; staging Technician is tech-view (button hidden)</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW - prod side unverified (no live prod data)</t>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>spec-predicted / NEEDS REVIEW - prod side unverified (no live prod data)</t>
         </is>
       </c>
     </row>
@@ -981,17 +1105,27 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Spec 'Behavior Changes for Migrating Users' table - Parts Manager: 'Loses WO Delete'</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Spec Behavior-Changes: Parts Manager 'Loses WO ... Delete'</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW - prod side unverified (no live prod data)</t>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>spec-predicted / NEEDS REVIEW - prod side unverified (no live prod data)</t>
         </is>
       </c>
     </row>
@@ -1028,17 +1162,27 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Spec 'Behavior Changes for Migrating Users' table - Parts Manager: 'Loses WO Lines Delete'</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Spec Behavior-Changes: Parts Manager 'Loses ... WOL Delete'</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW - prod side unverified (no live prod data)</t>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>spec-predicted / NEEDS REVIEW - prod side unverified (no live prod data)</t>
         </is>
       </c>
     </row>
@@ -1075,17 +1219,27 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Spec 'Behavior Changes for Migrating Users' table - Office: 'Catalog reduced to View only' (prod Office had Catalog Create&amp;Edit)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Spec Behavior-Changes: Office 'Catalog reduced to V only' (prod Office had Catalog Create&amp;Edit)</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW - prod side unverified (no live prod data)</t>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>spec-predicted / NEEDS REVIEW - prod side unverified (no live prod data)</t>
         </is>
       </c>
     </row>
@@ -1100,15 +1254,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1129,15 +1285,25 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t># spec-predicted PROD-only</t>
+          <t># prod&gt;staging deltas</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
+          <t># intended reductions (Yes)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t># NOT-in-spec reductions (No) = RELEASE RISK</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
           <t>Highest severity</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Needs-review</t>
         </is>
@@ -1162,12 +1328,18 @@
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>YES - all prod cells unverified</t>
         </is>
@@ -1192,12 +1364,18 @@
       <c r="D3" t="n">
         <v>5</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>YES - all prod cells unverified</t>
         </is>
@@ -1222,12 +1400,18 @@
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>YES - all prod cells unverified</t>
         </is>
@@ -1252,12 +1436,18 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>YES - all prod cells unverified</t>
         </is>
@@ -1282,12 +1472,18 @@
       <c r="D6" t="n">
         <v>1</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>YES - all prod cells unverified</t>
         </is>
@@ -1312,12 +1508,18 @@
       <c r="D7" t="n">
         <v>1</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>YES - all prod cells unverified</t>
         </is>
@@ -1342,12 +1544,18 @@
       <c r="D8" t="n">
         <v>2</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>YES - all prod cells unverified</t>
         </is>
@@ -1372,12 +1580,18 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>YES - all prod cells unverified</t>
         </is>
@@ -1402,12 +1616,18 @@
       <c r="D10" t="n">
         <v>1</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>YES - all prod cells unverified</t>
         </is>
@@ -1432,12 +1652,18 @@
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>YES - all prod cells unverified</t>
         </is>
@@ -1462,14 +1688,47 @@
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>YES - all prod cells unverified</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL (all roles)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>NOTE: 'No' (NOT-in-spec) reductions are the headline release risks. They are 0 in this INTERIM because every delta captured so far is a spec-DECLARED reduction (Yes). Live production capture may reveal prod&gt;staging gaps the spec does NOT account for (No) - add them with intended='No', spec_citation='not in spec'.</t>
         </is>
       </c>
     </row>
@@ -3617,7 +3876,7 @@
           <t>Production data NOT captured</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Production could not be authenticated. Missing a valid production sv_sso_session (64-hex). Every prod GET returned 409 'Session has expired'; dev quick-login returns 500 on prod. cf_clearance / Cloudflare is NOT the blocker (409 returns even with no cookies). Host confirmed: SPA app.shopview.com, API api.shopview.com. NEED: a valid production sv_sso_session cookie (and confirmation prod org UUID).</t>
         </is>
@@ -3629,7 +3888,7 @@
           <t>Naming trap</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Legacy 'Service Advisor' -&gt; staging 'Senior Service Advisor' (renamed+expanded); staging 'Service Advisor' comes from legacy 'SA Limited View'. Do NOT match on name.</t>
         </is>
@@ -3641,7 +3900,7 @@
           <t>Spec vs migration-case contradiction</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Section-3549 migration cases C26514/C26515 were authored as 1:1 same-name mappings, contradicting the authoritative spec migration table. NEEDS USER CONFIRMATION which is authoritative for the compare (recommend the spec table).</t>
         </is>
@@ -3653,7 +3912,7 @@
           <t>Prod role inventory unknown</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>The 15 legacy roles are the program-wide catalog; the target prod org may hold a subset and/or shop-specific custom roles. Enumerate live before mapping.</t>
         </is>
@@ -3665,7 +3924,7 @@
           <t>Prod permission representation unknown</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Old-model API shape not yet observed (fe-permissions route 404s on prod). Discover live: GET /api/roles/{id}, /api/auth/me, /api/staff/{id}.</t>
         </is>
@@ -3677,7 +3936,7 @@
           <t>Send-to-Terminal not in spec reduction list</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Send to Terminal (take-payment) is gated in staging on invoicingPaymentsCreateAndEdit AND customerPortalPageAccess. Not on the spec's 'Loses' list; must be diffed live per prod role once prod data is available.</t>
         </is>

</xml_diff>

<commit_message>
Custom Roles: finalize prod-vs-staging compare under QA-lead-confirmed mapping
Lock the confirmed role mapping (spec migration table authoritative, QA lead
2026-07-14): Senior Service Advisor <- Service Advisor + SA Technician + SA No
Reports; Service Advisor <- SA Limited View; Administrator compared 1:1 (Owner
N/A - no Owner role in either env). Clear the mapping-unconfirmed flag on the
Service-Advisor / Senior-SA rows (per-capability NEEDS-REVIEW preserved).
Recompute under the confirmed mapping changed no rows.

Headline counts unchanged: ALL STAGING-LESS No=52/Yes=4, STAGING-MORE No=53/
Yes=18; WO-granular STAGING-LESS No=22, STAGING-MORE No=24.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/custom-roles-run/Prod-vs-Staging-Permission-Gaps_2026-07-14.xlsx
+++ b/build/custom-roles-run/Prod-vs-Staging-Permission-Gaps_2026-07-14.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -614,36 +614,71 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Service Advisor &amp; Senior Service Advisor rows are flagged NEEDS-REVIEW (mapping</t>
+          <t>MAPPING CONFIRMED by QA lead 2026-07-14 (spec migration table is authoritative):</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  unconfirmed) per the naming trap: legacy 'Service Advisor' -&gt; staging 'Senior SA';</t>
+          <t xml:space="preserve">  Senior Service Advisor &lt;- Service Advisor + SA Technician + SA No Reports (3 merged);</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  staging 'Service Advisor' &lt;- legacy 'SA Limited View'. Computed under the spec map.</t>
+          <t xml:space="preserve">  Service Advisor &lt;- SA Limited View. The naming trap is RESOLVED - these rows are FINAL</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (no longer NEEDS-REVIEW for mapping; a per-capability NEEDS-REVIEW may still apply where</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TABS: 'Deltas - ALL (bi-dir)' whole-app | 'Work Orders - granular' WO-only |</t>
+          <t xml:space="preserve">  an old-model atom has no clean equivalent / is FE-gated).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
+        <is>
+          <t>Administrator compared 1:1 (prod Administrator &lt;-&gt; staging Administrator); the spec's</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  'Owner merged in' is not applicable - no Owner role exists in either environment</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (confirmed by QA lead 2026-07-14). Administrator delta rows stand as computed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TABS: 'Deltas - ALL (bi-dir)' whole-app | 'Work Orders - granular' WO-only |</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Summary tabs (per-role Yes/No 2x2) | Full capability matrix | Open questions.</t>
         </is>
@@ -1864,12 +1899,12 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=live | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=live | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>live + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>live</t>
         </is>
       </c>
     </row>
@@ -1921,12 +1956,12 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=live | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=live | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>live + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>live</t>
         </is>
       </c>
     </row>
@@ -1978,12 +2013,12 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2035,12 +2070,12 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2092,12 +2127,12 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=live | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=live | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>live + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>live</t>
         </is>
       </c>
     </row>
@@ -2149,12 +2184,12 @@
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2206,12 +2241,12 @@
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2263,12 +2298,12 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2320,12 +2355,12 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2377,12 +2412,12 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2434,12 +2469,12 @@
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - No Reports | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2491,12 +2526,12 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=live | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=live | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>live + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>live</t>
         </is>
       </c>
     </row>
@@ -2548,12 +2583,12 @@
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2605,12 +2640,12 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=live | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=live | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>live + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>live</t>
         </is>
       </c>
     </row>
@@ -2662,12 +2697,12 @@
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=live | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=live | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>live + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>live</t>
         </is>
       </c>
     </row>
@@ -2719,12 +2754,12 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=live | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=live | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>live + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>live</t>
         </is>
       </c>
     </row>
@@ -2776,12 +2811,12 @@
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2833,12 +2868,12 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2890,12 +2925,12 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: (none of mapped) | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -2947,12 +2982,12 @@
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -3004,12 +3039,12 @@
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -3061,12 +3096,12 @@
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -3118,12 +3153,12 @@
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -3175,12 +3210,12 @@
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -3232,12 +3267,12 @@
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -8446,12 +8481,12 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=live | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=live | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>live + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>live</t>
         </is>
       </c>
     </row>
@@ -8503,12 +8538,12 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA&lt;-&gt;SSA mapping NOT user-confirmed</t>
+          <t>prod holder: Service Advisor - Limited View | staging live | old-&gt;new map conf=NEEDS-REVIEW | SA/SSA merge mapping CONFIRMED by QA lead 2026-07-14</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW + NEEDS-REVIEW (mapping unconfirmed)</t>
+          <t>NEEDS-REVIEW</t>
         </is>
       </c>
     </row>
@@ -11020,7 +11055,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11059,7 +11094,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11098,7 +11133,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11172,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11176,7 +11211,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11215,7 +11250,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11254,7 +11289,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11293,7 +11328,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11332,7 +11367,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11371,7 +11406,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11410,7 +11445,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11528,7 +11563,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11567,7 +11602,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11606,7 +11641,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11645,7 +11680,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>NEEDS-REVIEW</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11684,7 +11719,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11723,7 +11758,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11762,7 +11797,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11801,7 +11836,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11840,7 +11875,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11879,7 +11914,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -11918,7 +11953,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -18491,24 +18526,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Service Advisor / Senior SA mapping UNCONFIRMED</t>
+          <t>Service Advisor / Senior SA mapping CONFIRMED (QA lead 2026-07-14)</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Naming trap: legacy 'Service Advisor' -&gt; staging 'Senior Service Advisor' (renamed+expanded); staging 'Service Advisor' comes from legacy 'SA Limited View'. Section-3549 migration cases C26514/C26515 were authored as 1:1 same-name mappings, contradicting the spec migration table. All Service-Advisor / Senior-Service-Advisor rows are flagged NEEDS-REVIEW; computed under the spec migration table. CONFIRM which authority governs before treating those deltas as final.</t>
+          <t>Naming trap RESOLVED by QA lead 2026-07-14 (spec migration table is authoritative): staging 'Senior Service Advisor' &lt;- legacy Service Advisor + SA Technician + SA No Reports (3 merged); staging 'Service Advisor' &lt;- legacy 'SA Limited View'. All Service-Advisor / Senior-Service-Advisor rows are FINAL - the mapping-unconfirmed flag is removed. (The section-3549 1:1 same-name migration cases C26514/C26515 are superseded by this ruling.) A per-capability NEEDS-REVIEW may still apply where an old-model atom has no clean equivalent / is FE-gated.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>'Owner' legacy role ABSENT in this prod org</t>
+          <t>Administrator compared 1:1 (Owner not applicable)</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Spec migration maps Owner+Administrator -&gt; Admin. The compared prod org (72b2cc90-...) has NO Owner role in GET /api/iam/list-roles (14 legacy roles, not 15). Admin is diffed against Administrator only. If any prod org still has an Owner role, re-run the compare there.</t>
+          <t>Administrator compared 1:1 (prod Administrator &lt;-&gt; staging Administrator); the spec's 'Owner merged in' is not applicable - no Owner role exists in either environment; confirmed by QA lead 2026-07-14. The Administrator delta rows stand as computed from the live Administrator-vs-Administrator capture (not incomplete).</t>
         </is>
       </c>
     </row>

</xml_diff>